<commit_message>
Another large overhaul. Many fixes
</commit_message>
<xml_diff>
--- a/data/bb-templates/gs-blue-owl.xlsx
+++ b/data/bb-templates/gs-blue-owl.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Template"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
   <si>
     <t>note_sort</t>
   </si>
@@ -87,31 +87,28 @@
     <t>Rated Included Investors</t>
   </si>
   <si>
-    <t>Rated Included</t>
+    <t>Included Investors (Rated)</t>
   </si>
   <si>
     <t>Non-Rated Included Investors</t>
   </si>
   <si>
-    <t>Non-Rated Included</t>
+    <t>Included Investors (Non-Rated)</t>
   </si>
   <si>
     <t>Designated Institutional Investors</t>
   </si>
   <si>
-    <t>Designated Institutional</t>
+    <t>Insitutional Designated Investors</t>
   </si>
   <si>
     <t>Designated PWM Investors</t>
   </si>
   <si>
-    <t>Designated PWM</t>
+    <t>PWM Designated Investors</t>
   </si>
   <si>
     <t>Excluded Investors</t>
-  </si>
-  <si>
-    <t>Ineligible Investors</t>
   </si>
   <si>
     <t>tab_sort</t>
@@ -197,7 +194,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,6 +205,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -241,13 +244,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -578,57 +581,57 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3">
         <v>7</v>
@@ -637,25 +640,25 @@
         <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H2" s="3">
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="3">
+        <v>6</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K2" s="3">
-        <v>6</v>
-      </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -685,22 +688,22 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
@@ -711,7 +714,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" s="3">
         <v>7</v>
@@ -720,10 +723,10 @@
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -742,7 +745,7 @@
     <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="36.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -759,7 +762,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -773,7 +776,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -787,7 +790,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -801,7 +804,7 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -815,7 +818,7 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -826,7 +829,7 @@
         <v>29</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>